<commit_message>
contact portal done successfully
</commit_message>
<xml_diff>
--- a/taha new login bot/templates/login_template.xlsx
+++ b/taha new login bot/templates/login_template.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="510" yWindow="555" windowWidth="2040" windowHeight="1245"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Username</t>
   </si>
@@ -22,28 +22,61 @@
     <t>Password</t>
   </si>
   <si>
-    <t>channellink@outlook.com</t>
-  </si>
-  <si>
-    <t>Abdul@999</t>
-  </si>
-  <si>
-    <t>samisaeid059@gmail.com</t>
-  </si>
-  <si>
-    <t>Saeid@999</t>
-  </si>
-  <si>
-    <t>farhatazizi@yahoo.com</t>
-  </si>
-  <si>
-    <t>Hasima@999</t>
+    <t>wagmafaizi@gmail.com</t>
+  </si>
+  <si>
+    <t>Wagma@999</t>
   </si>
   <si>
     <t>Walidnehwi01@gmail.com</t>
   </si>
   <si>
     <t>Fatimat@999</t>
+  </si>
+  <si>
+    <t>arashganji@yahoo.com</t>
+  </si>
+  <si>
+    <t>arash@999</t>
+  </si>
+  <si>
+    <t>mirzaieshugufa1213@gmail.com</t>
+  </si>
+  <si>
+    <t>Shugufa@999</t>
+  </si>
+  <si>
+    <t>yakuptrkglu@gmail.com</t>
+  </si>
+  <si>
+    <t>Yakup@999</t>
+  </si>
+  <si>
+    <t>jl2002rw@yahoo.fr</t>
+  </si>
+  <si>
+    <t>Masoodaanwar16@gmail.com</t>
+  </si>
+  <si>
+    <t>Masooda@999</t>
+  </si>
+  <si>
+    <t>arta_assadi@yahoo.ca</t>
+  </si>
+  <si>
+    <t>Arta@999</t>
+  </si>
+  <si>
+    <t>sonigee@msn.com</t>
+  </si>
+  <si>
+    <t>Lubna@999</t>
+  </si>
+  <si>
+    <t>Yusufselcuk994@gmail.com</t>
+  </si>
+  <si>
+    <t>yusuf@999</t>
   </si>
 </sst>
 </file>
@@ -61,10 +94,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -196,7 +226,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -231,7 +260,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -408,11 +436,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -455,7 +483,52 @@
         <v>9</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>